<commit_message>
Read an optional Session column from the students file
One file can now cover both sessions of a day: a Session column with
Morning or Evening (FN/AN, AM/PM also work). A roll number may appear once
per session; duplicates within a session and unknown session values get
row-numbered errors. Files without the column work as before. Adds helpers
to split students by session and list those writing in both sessions.
</commit_message>
<xml_diff>
--- a/samples/students-template.xlsx
+++ b/samples/students-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -406,6 +406,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -427,6 +428,9 @@
       <c r="F1" t="str">
         <v>Special Needs</v>
       </c>
+      <c r="G1" t="str">
+        <v>Session</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -447,6 +451,9 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -467,6 +474,9 @@
       <c r="F3" t="str">
         <v>Wheelchair</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -487,6 +497,9 @@
       <c r="F4" t="str">
         <v/>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -507,17 +520,20 @@
       <c r="F5" t="str">
         <v/>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -628,29 +644,48 @@
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>One row per student writing an exam in this session. Replace the example rows with your own.</v>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Session</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Optional: Morning or Evening (FN/AN and AM/PM also work). Fill it in to plan both sessions of a day from one file; leave the column out for a single session.</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Students writing the same Paper Code will never be seated next to each other (how strictly is chosen in the app).</v>
+        <v>One row per student writing an exam in this session. Replace the example rows with your own.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>You can also upload a CSV with the same column headers.</v>
+        <v>Students writing the same Paper Code will never be seated next to each other (how strictly is chosen in the app).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Session is optional: fill in Morning or Evening to plan both sessions of a day from one file (a student may then appear once per session).</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>You can also upload a CSV with the same column headers.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Privacy: SeatWise reads this file inside your browser. It is never uploaded to any server.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>